<commit_message>
Update question bank output links
</commit_message>
<xml_diff>
--- a/question-bank/CSS_Question_Bank.xlsx
+++ b/question-bank/CSS_Question_Bank.xlsx
@@ -68,7 +68,7 @@
     <t xml:space="preserve">&lt;div class="card"&gt;&lt;h2&gt;Course Title&lt;/h2&gt;&lt;p&gt;Short description&lt;/p&gt;&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q01-style-a-profile-card.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q01-style-a-profile-card.html</t>
   </si>
   <si>
     <t xml:space="preserve">2. Format Article Typography</t>
@@ -86,7 +86,7 @@
     <t xml:space="preserve">Use rem units for font sizes. Keep body text left aligned.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q02-format-article-typography.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q02-format-article-typography.html</t>
   </si>
   <si>
     <t xml:space="preserve">3. Create a Color Badge Set</t>
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Badge text must remain readable with sufficient contrast.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q03-create-a-color-badge-set.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q03-create-a-color-badge-set.html</t>
   </si>
   <si>
     <t xml:space="preserve">4. Apply the Box Model</t>
@@ -122,7 +122,7 @@
     <t xml:space="preserve">Cards must have equal width and visible borders.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q04-apply-the-box-model.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q04-apply-the-box-model.html</t>
   </si>
   <si>
     <t xml:space="preserve">5. Style a Login Form</t>
@@ -140,7 +140,7 @@
     <t xml:space="preserve">Do not use JavaScript. Keep fields full width inside the form.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q05-style-a-login-form.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q05-style-a-login-form.html</t>
   </si>
   <si>
     <t xml:space="preserve">6. Add Background Effects</t>
@@ -158,7 +158,7 @@
     <t xml:space="preserve">The heading must remain visible over the background.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q06-add-background-effects.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q06-add-background-effects.html</t>
   </si>
   <si>
     <t xml:space="preserve">7. Build a Navigation Bar</t>
@@ -176,7 +176,7 @@
     <t xml:space="preserve">Nav links must have consistent spacing and no underline by default.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q07-build-a-navigation-bar.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q07-build-a-navigation-bar.html</t>
   </si>
   <si>
     <t xml:space="preserve">8. Design a Product Tile</t>
@@ -194,7 +194,7 @@
     <t xml:space="preserve">Avoid using !important.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q08-design-a-product-tile.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q08-design-a-product-tile.html</t>
   </si>
   <si>
     <t xml:space="preserve">9. Normalize Page Spacing</t>
@@ -212,7 +212,7 @@
     <t xml:space="preserve">Do not remove focus outlines.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q09-normalize-page-spacing.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q09-normalize-page-spacing.html</t>
   </si>
   <si>
     <t xml:space="preserve">10. Create Text Utility Classes</t>
@@ -230,7 +230,7 @@
     <t xml:space="preserve">Each utility class must do one job only.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q10-create-text-utility-classes.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q10-create-text-utility-classes.html</t>
   </si>
   <si>
     <t xml:space="preserve">CSS Layout Systems</t>
@@ -254,7 +254,7 @@
     <t xml:space="preserve">&lt;section class="layout-challenge"&gt;&lt;div&gt;Item 1&lt;/div&gt;&lt;div&gt;Item 2&lt;/div&gt;&lt;div&gt;Item 3&lt;/div&gt;&lt;/section&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q11-flex-navbar-alignment.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q11-flex-navbar-alignment.html</t>
   </si>
   <si>
     <t xml:space="preserve">2. Responsive Card Row</t>
@@ -272,7 +272,7 @@
     <t xml:space="preserve">Cards must not overlap when the viewport is narrow.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q12-responsive-card-row.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q12-responsive-card-row.html</t>
   </si>
   <si>
     <t xml:space="preserve">3. Two Column Portfolio Layout</t>
@@ -290,7 +290,7 @@
     <t xml:space="preserve">At desktop width, text must appear before image.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q13-two-column-portfolio-layout.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q13-two-column-portfolio-layout.html</t>
   </si>
   <si>
     <t xml:space="preserve">4. Analytics Dashboard Grid</t>
@@ -308,7 +308,7 @@
     <t xml:space="preserve">Sidebar must keep a fixed width on desktop.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q14-analytics-dashboard-grid.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q14-analytics-dashboard-grid.html</t>
   </si>
   <si>
     <t xml:space="preserve">5. Absolute Badge Position</t>
@@ -326,7 +326,7 @@
     <t xml:space="preserve">Badge must stay inside the card boundary.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q15-absolute-badge-position.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q15-absolute-badge-position.html</t>
   </si>
   <si>
     <t xml:space="preserve">6. Sticky Section Header</t>
@@ -344,7 +344,7 @@
     <t xml:space="preserve">Toolbar must not cover the first row.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q16-sticky-section-header.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q16-sticky-section-header.html</t>
   </si>
   <si>
     <t xml:space="preserve">7. Fixed Support Button</t>
@@ -362,7 +362,7 @@
     <t xml:space="preserve">Button must remain visible above page content.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q17-fixed-support-button.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q17-fixed-support-button.html</t>
   </si>
   <si>
     <t xml:space="preserve">8. Layered Modal Overlay</t>
@@ -380,7 +380,7 @@
     <t xml:space="preserve">Modal must appear above overlay.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q18-layered-modal-overlay.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q18-layered-modal-overlay.html</t>
   </si>
   <si>
     <t xml:space="preserve">9. Grid Gallery Layout</t>
@@ -398,7 +398,7 @@
     <t xml:space="preserve">Gallery items must keep equal gaps.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q19-grid-gallery-layout.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q19-grid-gallery-layout.html</t>
   </si>
   <si>
     <t xml:space="preserve">10. Flex Form Controls</t>
@@ -416,7 +416,7 @@
     <t xml:space="preserve">Input should take remaining width.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q20-flex-form-controls.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q20-flex-form-controls.html</t>
   </si>
   <si>
     <t xml:space="preserve">Responsive Web Design</t>
@@ -441,7 +441,7 @@
 HTML: Provided responsive component markup</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q21-mobile-first-navbar.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q21-mobile-first-navbar.html</t>
   </si>
   <si>
     <t xml:space="preserve">2. Responsive Card Grid</t>
@@ -459,7 +459,7 @@
     <t xml:space="preserve">Must start as one column on small screens.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q22-responsive-card-grid.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q22-responsive-card-grid.html</t>
   </si>
   <si>
     <t xml:space="preserve">3. Fluid Hero Sizing</t>
@@ -477,7 +477,7 @@
     <t xml:space="preserve">Do not use fixed pixel widths for the main container.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q23-fluid-hero-sizing.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q23-fluid-hero-sizing.html</t>
   </si>
   <si>
     <t xml:space="preserve">4. Responsive Form Layout</t>
@@ -495,7 +495,7 @@
     <t xml:space="preserve">Labels must stay above their fields.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q24-responsive-form-layout.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q24-responsive-form-layout.html</t>
   </si>
   <si>
     <t xml:space="preserve">5. Adaptive Dashboard Panels</t>
@@ -513,7 +513,7 @@
     <t xml:space="preserve">Widgets must preserve readable spacing.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q25-adaptive-dashboard-panels.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q25-adaptive-dashboard-panels.html</t>
   </si>
   <si>
     <t xml:space="preserve">6. Responsive Image Treatment</t>
@@ -531,7 +531,7 @@
     <t xml:space="preserve">Images must not overflow their containers.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q26-responsive-image-treatment.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q26-responsive-image-treatment.html</t>
   </si>
   <si>
     <t xml:space="preserve">7. Viewport Based Split Section</t>
@@ -549,7 +549,7 @@
     <t xml:space="preserve">Mobile content must not be clipped.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q27-viewport-based-split-section.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q27-viewport-based-split-section.html</t>
   </si>
   <si>
     <t xml:space="preserve">8. Responsive Table Alternative</t>
@@ -567,7 +567,7 @@
     <t xml:space="preserve">Each mobile row must show label and value.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q28-responsive-table-alternative.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q28-responsive-table-alternative.html</t>
   </si>
   <si>
     <t xml:space="preserve">9. Scalable Spacing System</t>
@@ -585,7 +585,7 @@
     <t xml:space="preserve">Avoid hardcoding repeated pixel spacing.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q29-scalable-spacing-system.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q29-scalable-spacing-system.html</t>
   </si>
   <si>
     <t xml:space="preserve">10. Accessible Responsive Footer</t>
@@ -603,7 +603,7 @@
     <t xml:space="preserve">Link tap targets must be at least 44px high on mobile.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q30-accessible-responsive-footer.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q30-accessible-responsive-footer.html</t>
   </si>
   <si>
     <t xml:space="preserve">Tailwind CSS</t>
@@ -627,7 +627,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-profile-card"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q31-tailwind-profile-card.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q31-tailwind-profile-card.html</t>
   </si>
   <si>
     <t xml:space="preserve">2. Tailwind Responsive Navbar</t>
@@ -648,7 +648,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-responsive-navbar"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q32-tailwind-responsive-navbar.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q32-tailwind-responsive-navbar.html</t>
   </si>
   <si>
     <t xml:space="preserve">3. Tailwind Course Grid</t>
@@ -669,7 +669,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-course-grid"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q33-tailwind-course-grid.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q33-tailwind-course-grid.html</t>
   </si>
   <si>
     <t xml:space="preserve">4. Tailwind Button States</t>
@@ -690,7 +690,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-button-states"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q34-tailwind-button-states.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q34-tailwind-button-states.html</t>
   </si>
   <si>
     <t xml:space="preserve">5. Tailwind Form Panel</t>
@@ -711,7 +711,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-form-panel"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q35-tailwind-form-panel.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q35-tailwind-form-panel.html</t>
   </si>
   <si>
     <t xml:space="preserve">6. Tailwind Sidebar Layout</t>
@@ -732,7 +732,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-sidebar-layout"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q36-tailwind-sidebar-layout.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q36-tailwind-sidebar-layout.html</t>
   </si>
   <si>
     <t xml:space="preserve">7. Tailwind Theme Color Usage</t>
@@ -753,7 +753,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-theme-color-usage"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q37-tailwind-theme-color-usage.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q37-tailwind-theme-color-usage.html</t>
   </si>
   <si>
     <t xml:space="preserve">8. Tailwind Spacing System</t>
@@ -774,7 +774,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-spacing-system"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q38-tailwind-spacing-system.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q38-tailwind-spacing-system.html</t>
   </si>
   <si>
     <t xml:space="preserve">9. Tailwind Dashboard Widgets</t>
@@ -795,7 +795,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-dashboard-widgets"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q39-tailwind-dashboard-widgets.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q39-tailwind-dashboard-widgets.html</t>
   </si>
   <si>
     <t xml:space="preserve">10. Tailwind Production Component</t>
@@ -816,7 +816,7 @@
     <t xml:space="preserve">&lt;div class="challenge tailwind-production-component"&gt;Apply Tailwind classes to match the requested UI.&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q40-tailwind-production-component.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q40-tailwind-production-component.html</t>
   </si>
   <si>
     <t xml:space="preserve">UI Design Concepts</t>
@@ -841,7 +841,7 @@
 &lt;div class="panel"&gt;Dashboard content&lt;/div&gt;</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q41-hoverable-dashboard-card.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q41-hoverable-dashboard-card.html</t>
   </si>
   <si>
     <t xml:space="preserve">2. Animated Submit Button</t>
@@ -859,7 +859,7 @@
     <t xml:space="preserve">Disabled state must look inactive and block pointer styling.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q42-animated-submit-button.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q42-animated-submit-button.html</t>
   </si>
   <si>
     <t xml:space="preserve">3. Skeleton Loading Card</t>
@@ -877,7 +877,7 @@
     <t xml:space="preserve">Animation should be smooth and not distract users.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q43-skeleton-loading-card.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q43-skeleton-loading-card.html</t>
   </si>
   <si>
     <t xml:space="preserve">4. Sidebar Navigation States</t>
@@ -895,7 +895,7 @@
     <t xml:space="preserve">Active state must differ from hover state.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q44-sidebar-navigation-states.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q44-sidebar-navigation-states.html</t>
   </si>
   <si>
     <t xml:space="preserve">5. Interactive Form Feedback</t>
@@ -913,7 +913,7 @@
     <t xml:space="preserve">Invalid state must not rely only on color.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q45-interactive-form-feedback.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q45-interactive-form-feedback.html</t>
   </si>
   <si>
     <t xml:space="preserve">6. Card Widget Hierarchy</t>
@@ -931,7 +931,7 @@
     <t xml:space="preserve">The metric value must be the most prominent element.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q46-card-widget-hierarchy.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q46-card-widget-hierarchy.html</t>
   </si>
   <si>
     <t xml:space="preserve">7. Fade In Content Section</t>
@@ -949,7 +949,7 @@
     <t xml:space="preserve">Animation duration must be under 500ms.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q47-fade-in-content-section.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q47-fade-in-content-section.html</t>
   </si>
   <si>
     <t xml:space="preserve">8. Accessible Tooltip Styling</t>
@@ -967,7 +967,7 @@
     <t xml:space="preserve">Tooltip must work with keyboard focus.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q48-accessible-tooltip-styling.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q48-accessible-tooltip-styling.html</t>
   </si>
   <si>
     <t xml:space="preserve">9. Interactive Modal Motion</t>
@@ -985,7 +985,7 @@
     <t xml:space="preserve">Respect reduced motion with a media query.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q49-interactive-modal-motion.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q49-interactive-modal-motion.html</t>
   </si>
   <si>
     <t xml:space="preserve">10. Empty State Panel</t>
@@ -1003,7 +1003,7 @@
     <t xml:space="preserve">The action button must remain visually prominent.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q50-empty-state-panel.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q50-empty-state-panel.html</t>
   </si>
   <si>
     <t xml:space="preserve">Production-Level Frontend Styling</t>
@@ -1027,7 +1027,7 @@
     <t xml:space="preserve">Existing component classes and semantic HTML from a React frontend</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q51-reusable-component-classes.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q51-reusable-component-classes.html</t>
   </si>
   <si>
     <t xml:space="preserve">2. Organized CSS Structure</t>
@@ -1045,7 +1045,7 @@
     <t xml:space="preserve">Keep selectors readable and avoid deep nesting.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q52-organized-css-structure.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q52-organized-css-structure.html</t>
   </si>
   <si>
     <t xml:space="preserve">3. CSS Variables Theme</t>
@@ -1063,7 +1063,7 @@
     <t xml:space="preserve">Components must use variables instead of hardcoded colors.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q53-css-variables-theme.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q53-css-variables-theme.html</t>
   </si>
   <si>
     <t xml:space="preserve">4. Accessible Contrast Fix</t>
@@ -1081,7 +1081,7 @@
     <t xml:space="preserve">Do not reduce font size to solve layout issues.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q54-accessible-contrast-fix.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q54-accessible-contrast-fix.html</t>
   </si>
   <si>
     <t xml:space="preserve">5. Production Form Component</t>
@@ -1099,7 +1099,7 @@
     <t xml:space="preserve">Error text must be visible and associated with the field visually.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q55-production-form-component.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q55-production-form-component.html</t>
   </si>
   <si>
     <t xml:space="preserve">6. Optimize CSS Asset Usage</t>
@@ -1117,7 +1117,7 @@
     <t xml:space="preserve">Do not remove required brand visuals.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q56-optimize-css-asset-usage.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q56-optimize-css-asset-usage.html</t>
   </si>
   <si>
     <t xml:space="preserve">7. Component Scoped Naming</t>
@@ -1135,7 +1135,7 @@
     <t xml:space="preserve">Class names must communicate component ownership.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q57-component-scoped-naming.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q57-component-scoped-naming.html</t>
   </si>
   <si>
     <t xml:space="preserve">8. Production Dashboard Layout</t>
@@ -1153,7 +1153,7 @@
     <t xml:space="preserve">The shell must remain usable on mobile.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q58-production-dashboard-layout.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q58-production-dashboard-layout.html</t>
   </si>
   <si>
     <t xml:space="preserve">9. Semantic UI Styling</t>
@@ -1171,7 +1171,7 @@
     <t xml:space="preserve">Do not remove outlines or hide labels.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q59-semantic-ui-styling.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q59-semantic-ui-styling.html</t>
   </si>
   <si>
     <t xml:space="preserve">10. Performance Friendly Animation</t>
@@ -1189,7 +1189,7 @@
     <t xml:space="preserve">Avoid animating width, height, top, or left.</t>
   </si>
   <si>
-    <t xml:space="preserve">https://nithya-sri-14.github.io/css-beginner/question-bank/outputs/q60-performance-friendly-animation.html</t>
+    <t xml:space="preserve">https://htmlpreview.github.io/?https://github.com/Nithya-sri-14/css-beginner/blob/main/question-bank/outputs/q60-performance-friendly-animation.html</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update unique hints and constraints
</commit_message>
<xml_diff>
--- a/question-bank/CSS_Question_Bank.xlsx
+++ b/question-bank/CSS_Question_Bank.xlsx
@@ -604,12 +604,12 @@
       </c>
       <c r="G2" s="4" t="inlineStr">
         <is>
-          <t>Target the provided class names and avoid inline styles.</t>
+          <t>Inspect the provided markup for 'Style a Profile Card', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H2" s="4" t="inlineStr">
         <is>
-          <t>Use only CSS3. Do not change the HTML structure.</t>
+          <t>Do not change the provided HTML structure for 'Style a Profile Card'. The submitted CSS must match the sample output for question 1 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I2" s="4" t="inlineStr">
@@ -656,12 +656,12 @@
       </c>
       <c r="G3" s="6" t="inlineStr">
         <is>
-          <t>Style headings and paragraphs with separate selectors.</t>
+          <t>Style the form controls for 'Format Article Typography' in their normal and focus states; labels, inputs, helper text, and buttons should remain aligned and readable.</t>
         </is>
       </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
-          <t>Use rem units for font sizes. Keep body text left aligned.</t>
+          <t>Do not change the provided HTML structure for 'Format Article Typography'. Inputs must remain keyboard focusable, labels must remain visible, and focus styling must not be removed.</t>
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr">
@@ -708,12 +708,12 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Create reusable badge classes and one modifier class per state.</t>
+          <t>Set the correct positioning context for 'Create a Color Badge Set' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>Badge text must remain readable with sufficient contrast.</t>
+          <t>Do not change the provided HTML structure for 'Create a Color Badge Set'. The positioned element must stay inside or above the intended parent area and must not overlap unrelated content.</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
@@ -760,12 +760,12 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Set box-sizing globally and style the card class.</t>
+          <t>Inspect the provided markup for 'Apply the Box Model', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
-          <t>Cards must have equal width and visible borders.</t>
+          <t>Do not change the provided HTML structure for 'Apply the Box Model'. The submitted CSS must match the sample output for question 4 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>Use input[type='text'], input[type='password'], and button selectors.</t>
+          <t>Style the form controls for 'Style a Login Form' in their normal and focus states; labels, inputs, helper text, and buttons should remain aligned and readable.</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t>Do not use JavaScript. Keep fields full width inside the form.</t>
+          <t>Do not change the provided HTML structure for 'Style a Login Form'. Inputs must remain keyboard focusable, labels must remain visible, and focus styling must not be removed.</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Use a gradient overlay and readable text color.</t>
+          <t>Inspect the provided markup for 'Add Background Effects', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>The heading must remain visible over the background.</t>
+          <t>Do not change the provided HTML structure for 'Add Background Effects'. The submitted CSS must match the sample output for question 6 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Remove list styles and style anchor hover states.</t>
+          <t>Inspect the provided markup for 'Build a Navigation Bar', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t>Nav links must have consistent spacing and no underline by default.</t>
+          <t>Do not change the provided HTML structure for 'Build a Navigation Bar'. The submitted CSS must match the sample output for question 7 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -968,12 +968,12 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>Use the ID for the featured tile and classes for shared styles.</t>
+          <t>Inspect the provided markup for 'Design a Product Tile', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
-          <t>Avoid using !important.</t>
+          <t>Do not change the provided HTML structure for 'Design a Product Tile'. The submitted CSS must match the sample output for question 8 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -1020,12 +1020,12 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>Apply a minimal reset before component styles.</t>
+          <t>Inspect the provided markup for 'Normalize Page Spacing', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t>Do not remove focus outlines.</t>
+          <t>Do not change the provided HTML structure for 'Normalize Page Spacing'. The submitted CSS must match the sample output for question 9 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1072,12 +1072,12 @@
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Create one class per utility.</t>
+          <t>Focus on text hierarchy for 'Create Text Utility Classes': set font family, size, weight, line-height, spacing, and color to match the target output.</t>
         </is>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
-          <t>Each utility class must do one job only.</t>
+          <t>Do not change the provided HTML structure for 'Create Text Utility Classes'. Use rem or relative units for text sizing where appropriate; do not use viewport-width font sizing or clipped single-line text.</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -1124,12 +1124,12 @@
       </c>
       <c r="G12" s="4" t="inlineStr">
         <is>
-          <t>Use element selectors and avoid inline styles.</t>
+          <t>Focus on text hierarchy for 'Style Heading Levels': set font family, size, weight, line-height, spacing, and color to match the target output.</t>
         </is>
       </c>
       <c r="H12" s="4" t="inlineStr">
         <is>
-          <t>Each heading level must look visually distinct.</t>
+          <t>Do not change the provided HTML structure for 'Style Heading Levels'. Use rem or relative units for text sizing where appropriate; do not use viewport-width font sizing or clipped single-line text.</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
@@ -1176,12 +1176,12 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Use anchor pseudo-classes in a logical order.</t>
+          <t>Inspect the provided markup for 'Create Link Styles', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>Do not remove keyboard focus visibility.</t>
+          <t>Do not change the provided HTML structure for 'Create Link Styles'. The submitted CSS must match the sample output for question 12 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -1228,12 +1228,12 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>Use one base alert class and modifier classes.</t>
+          <t>Choose foreground, background, and border colors for 'Build Alert Boxes' so every state is visually distinct and the text stays readable.</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t>Each alert must include padding, border, and readable colors.</t>
+          <t>Do not change the provided HTML structure for 'Build Alert Boxes'. Each visual state must include readable text contrast and at least one non-color cue such as a border, label, icon, or spacing difference.</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1280,12 +1280,12 @@
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Use font-family with multiple fallbacks.</t>
+          <t>Focus on text hierarchy for 'Use Font Families Correctly': set font family, size, weight, line-height, spacing, and color to match the target output.</t>
         </is>
       </c>
       <c r="H15" s="6" t="inlineStr">
         <is>
-          <t>Code text must use a monospace stack.</t>
+          <t>Do not change the provided HTML structure for 'Use Font Families Correctly'. Use rem or relative units for text sizing where appropriate; do not use viewport-width font sizing or clipped single-line text.</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -1332,12 +1332,12 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>Use margin auto for horizontal centering.</t>
+          <t>Inspect the provided markup for 'Control Element Widths', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t>Container width must remain responsive.</t>
+          <t>Do not change the provided HTML structure for 'Control Element Widths'. The submitted CSS must match the sample output for question 15 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
@@ -1384,12 +1384,12 @@
       </c>
       <c r="G17" s="6" t="inlineStr">
         <is>
-          <t>Use class selectors for each border type.</t>
+          <t>Inspect the provided markup for 'Add Border Variations', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
         <is>
-          <t>Borders must not change the page layout unexpectedly.</t>
+          <t>Do not change the provided HTML structure for 'Add Border Variations'. The submitted CSS must match the sample output for question 16 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1436,12 +1436,12 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>Use different radius values based on component shape.</t>
+          <t>Inspect the provided markup for 'Apply Rounded Corners', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t>Avatar must appear circular.</t>
+          <t>Do not change the provided HTML structure for 'Apply Rounded Corners'. The submitted CSS must match the sample output for question 17 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
@@ -1488,12 +1488,12 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Use opacity only where it does not harm readability.</t>
+          <t>Inspect the provided markup for 'Practice Opacity', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>Main text must remain fully readable.</t>
+          <t>Do not change the provided HTML structure for 'Practice Opacity'. The submitted CSS must match the sample output for question 18 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
@@ -1540,12 +1540,12 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>Group selectors that share the same declarations.</t>
+          <t>Inspect the provided markup for 'Group Shared Selectors', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t>Do not group selectors with different behavior.</t>
+          <t>Do not change the provided HTML structure for 'Group Shared Selectors'. The submitted CSS must match the sample output for question 19 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
@@ -1592,12 +1592,12 @@
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>Keep each utility class focused on one property.</t>
+          <t>Inspect the provided markup for 'Create Simple Utility Classes', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>Do not combine unrelated styles in one utility.</t>
+          <t>Do not change the provided HTML structure for 'Create Simple Utility Classes'. The submitted CSS must match the sample output for question 20 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -1644,12 +1644,12 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>Use justify-content and align-items on the navbar container.</t>
+          <t>Use Flexbox for 'Flex Navbar Alignment' and control alignment with justify-content, align-items, gap, flex-wrap, or flex-grow based on the target output.</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
         <is>
-          <t>Do not use floats. Keep the logo on the left and button on the right.</t>
+          <t>Do not change the provided HTML structure for 'Flex Navbar Alignment'. Use Flexbox for the main alignment; avoid floats, negative margins, and fixed pixel offsets for primary positioning.</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -1696,12 +1696,12 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Use flex-wrap and gap.</t>
+          <t>Start from the smallest screen layout for 'Responsive Card Row', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H23" s="6" t="inlineStr">
         <is>
-          <t>Cards must not overlap when the viewport is narrow.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Card Row'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -1748,12 +1748,12 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>Use grid-template-columns and align-items.</t>
+          <t>Inspect the provided markup for 'Two Column Portfolio Layout', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t>At desktop width, text must appear before image.</t>
+          <t>Do not change the provided HTML structure for 'Two Column Portfolio Layout'. The submitted CSS must match the sample output for question 23 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
@@ -1800,12 +1800,12 @@
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Name grid areas clearly.</t>
+          <t>Use CSS Grid properties for 'Analytics Dashboard Grid', especially grid-template-columns, gap, and responsive track sizing where the target output shows structured rows or columns.</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>Sidebar must keep a fixed width on desktop.</t>
+          <t>Do not change the provided HTML structure for 'Analytics Dashboard Grid'. Use CSS Grid for the main arrangement; do not solve the layout with floats, HTML tables, or fixed absolute positions.</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -1852,12 +1852,12 @@
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>Set the card to relative and the badge to absolute.</t>
+          <t>Set the correct positioning context for 'Absolute Badge Position' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t>Badge must stay inside the card boundary.</t>
+          <t>Do not change the provided HTML structure for 'Absolute Badge Position'. The positioned element must stay inside or above the intended parent area and must not overlap unrelated content.</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
@@ -1904,12 +1904,12 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>Use position: sticky with a top offset.</t>
+          <t>Set the correct positioning context for 'Sticky Section Header' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>Toolbar must not cover the first row.</t>
+          <t>Do not change the provided HTML structure for 'Sticky Section Header'. Use position: sticky with an explicit top value; the sticky element must not hide the first content row.</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -1956,12 +1956,12 @@
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>Use position: fixed and z-index.</t>
+          <t>Set the correct positioning context for 'Fixed Support Button' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H28" s="4" t="inlineStr">
         <is>
-          <t>Button must remain visible above page content.</t>
+          <t>Do not change the provided HTML structure for 'Fixed Support Button'. Use position: fixed for the persistent action; it must remain visible above page content without blocking important text.</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
@@ -2008,12 +2008,12 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Create separate overlay and modal layers.</t>
+          <t>Set the correct positioning context for 'Layered Modal Overlay' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>Modal must appear above overlay.</t>
+          <t>Do not change the provided HTML structure for 'Layered Modal Overlay'. The overlay must sit below the dialog, the dialog must remain visible above the overlay, and the page content must not visually cover the modal.</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -2060,12 +2060,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>Use repeat(auto-fit, minmax()).</t>
+          <t>Use CSS Grid properties for 'Grid Gallery Layout', especially grid-template-columns, gap, and responsive track sizing where the target output shows structured rows or columns.</t>
         </is>
       </c>
       <c r="H30" s="4" t="inlineStr">
         <is>
-          <t>Gallery items must keep equal gaps.</t>
+          <t>Do not change the provided HTML structure for 'Grid Gallery Layout'. Use CSS Grid for the main arrangement; do not solve the layout with floats, HTML tables, or fixed absolute positions.</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -2112,12 +2112,12 @@
       </c>
       <c r="G31" s="6" t="inlineStr">
         <is>
-          <t>Use flex-basis or flex-grow for the input.</t>
+          <t>Use Flexbox for 'Flex Form Controls' and control alignment with justify-content, align-items, gap, flex-wrap, or flex-grow based on the target output.</t>
         </is>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>Input should take remaining width.</t>
+          <t>Do not change the provided HTML structure for 'Flex Form Controls'. Use Flexbox for the main alignment; avoid floats, negative margins, and fixed pixel offsets for primary positioning.</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -2164,12 +2164,12 @@
       </c>
       <c r="G32" s="4" t="inlineStr">
         <is>
-          <t>Apply display flex to the parent container.</t>
+          <t>Use Flexbox for 'Center Content With Flexbox' and control alignment with justify-content, align-items, gap, flex-wrap, or flex-grow based on the target output.</t>
         </is>
       </c>
       <c r="H32" s="4" t="inlineStr">
         <is>
-          <t>Do not use absolute positioning.</t>
+          <t>Do not change the provided HTML structure for 'Center Content With Flexbox'. Use Flexbox for the main alignment; avoid floats, negative margins, and fixed pixel offsets for primary positioning.</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -2216,12 +2216,12 @@
       </c>
       <c r="G33" s="6" t="inlineStr">
         <is>
-          <t>Use flex: 1 on child items.</t>
+          <t>Inspect the provided markup for 'Build Equal Width Columns', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>Columns must keep equal width on desktop.</t>
+          <t>Do not change the provided HTML structure for 'Build Equal Width Columns'. The submitted CSS must match the sample output for question 32 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -2268,12 +2268,12 @@
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>Use grid-template-columns and gap.</t>
+          <t>Use CSS Grid properties for 'Create a Simple Grid', especially grid-template-columns, gap, and responsive track sizing where the target output shows structured rows or columns.</t>
         </is>
       </c>
       <c r="H34" s="4" t="inlineStr">
         <is>
-          <t>No floats or table layout allowed.</t>
+          <t>Do not change the provided HTML structure for 'Create a Simple Grid'. Use CSS Grid for the main arrangement; do not solve the layout with floats, HTML tables, or fixed absolute positions.</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -2320,12 +2320,12 @@
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>Use Flexbox alignment and gap.</t>
+          <t>Inspect the provided markup for 'Make a Header Layout', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>Search box should take available space.</t>
+          <t>Do not change the provided HTML structure for 'Make a Header Layout'. The submitted CSS must match the sample output for question 34 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -2372,12 +2372,12 @@
       </c>
       <c r="G36" s="4" t="inlineStr">
         <is>
-          <t>Set the notice container to position relative.</t>
+          <t>Set the correct positioning context for 'Position a Close Icon' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H36" s="4" t="inlineStr">
         <is>
-          <t>The icon must remain inside the notice box.</t>
+          <t>Do not change the provided HTML structure for 'Position a Close Icon'. The positioned element must stay inside or above the intended parent area and must not overlap unrelated content.</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -2424,12 +2424,12 @@
       </c>
       <c r="G37" s="6" t="inlineStr">
         <is>
-          <t>Use position sticky and top.</t>
+          <t>Use Flexbox for 'Create a Sticky Navbar' and control alignment with justify-content, align-items, gap, flex-wrap, or flex-grow based on the target output.</t>
         </is>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>Navbar must remain above page content.</t>
+          <t>Do not change the provided HTML structure for 'Create a Sticky Navbar'. Use Flexbox for the main alignment; avoid floats, negative margins, and fixed pixel offsets for primary positioning.</t>
         </is>
       </c>
       <c r="I37" s="6" t="inlineStr">
@@ -2476,12 +2476,12 @@
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>Use gap instead of margin hacks.</t>
+          <t>Inspect the provided markup for 'Stack Cards With Gap', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H38" s="4" t="inlineStr">
         <is>
-          <t>Spacing between all cards must be equal.</t>
+          <t>Do not change the provided HTML structure for 'Stack Cards With Gap'. The submitted CSS must match the sample output for question 37 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -2528,12 +2528,12 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>Use grid-template-columns.</t>
+          <t>Use CSS Grid properties for 'Create Grid Sidebar Layout', especially grid-template-columns, gap, and responsive track sizing where the target output shows structured rows or columns.</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>Sidebar must stay narrower than main content.</t>
+          <t>Do not change the provided HTML structure for 'Create Grid Sidebar Layout'. Use CSS Grid for the main arrangement; do not solve the layout with floats, HTML tables, or fixed absolute positions.</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -2580,12 +2580,12 @@
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Use positioned elements before z-index.</t>
+          <t>Set the correct positioning context for 'Control Z Index Layers' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H40" s="4" t="inlineStr">
         <is>
-          <t>Dropdown must appear above the page cards.</t>
+          <t>Do not change the provided HTML structure for 'Control Z Index Layers'. The positioned element must stay inside or above the intended parent area and must not overlap unrelated content.</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -2632,12 +2632,12 @@
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>Use justify-content space-between.</t>
+          <t>Use Flexbox for 'Align Items in a Toolbar' and control alignment with justify-content, align-items, gap, flex-wrap, or flex-grow based on the target output.</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>Toolbar items must remain vertically centered.</t>
+          <t>Do not change the provided HTML structure for 'Align Items in a Toolbar'. Use Flexbox for the main alignment; avoid floats, negative margins, and fixed pixel offsets for primary positioning.</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -2684,12 +2684,12 @@
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Write base mobile styles first, then add a media query.</t>
+          <t>Start from the smallest screen layout for 'Mobile First Navbar', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H42" s="4" t="inlineStr">
         <is>
-          <t>Use @media (min-width: 768px).</t>
+          <t>Do not change the provided HTML structure for 'Mobile First Navbar'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -2737,12 +2737,12 @@
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>Use CSS Grid and media queries.</t>
+          <t>Start from the smallest screen layout for 'Responsive Card Grid', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>Must start as one column on small screens.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Card Grid'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -2790,12 +2790,12 @@
       </c>
       <c r="G44" s="4" t="inlineStr">
         <is>
-          <t>Use min-height and max-width constraints.</t>
+          <t>Inspect the provided markup for 'Fluid Hero Sizing', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H44" s="4" t="inlineStr">
         <is>
-          <t>Do not use fixed pixel widths for the main container.</t>
+          <t>Do not change the provided HTML structure for 'Fluid Hero Sizing'. The submitted CSS must match the sample output for question 43 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -2843,12 +2843,12 @@
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>Use grid or flex with a breakpoint.</t>
+          <t>Start from the smallest screen layout for 'Responsive Form Layout', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>Labels must stay above their fields.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Form Layout'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -2896,12 +2896,12 @@
       </c>
       <c r="G46" s="4" t="inlineStr">
         <is>
-          <t>Define breakpoints for tablet and desktop.</t>
+          <t>Inspect the provided markup for 'Adaptive Dashboard Panels', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H46" s="4" t="inlineStr">
         <is>
-          <t>Widgets must preserve readable spacing.</t>
+          <t>Do not change the provided HTML structure for 'Adaptive Dashboard Panels'. The submitted CSS must match the sample output for question 45 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -2949,12 +2949,12 @@
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>Use max-width, height:auto, and object-fit where needed.</t>
+          <t>Start from the smallest screen layout for 'Responsive Image Treatment', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>Images must not overflow their containers.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Image Treatment'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
@@ -3002,12 +3002,12 @@
       </c>
       <c r="G48" s="4" t="inlineStr">
         <is>
-          <t>Use vh carefully and override it in a media query.</t>
+          <t>Start from the smallest screen layout for 'Viewport Based Split Section', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H48" s="4" t="inlineStr">
         <is>
-          <t>Mobile content must not be clipped.</t>
+          <t>Do not change the provided HTML structure for 'Viewport Based Split Section'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -3055,12 +3055,12 @@
       </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
-          <t>Use CSS display changes inside a max-width media query.</t>
+          <t>Start from the smallest screen layout for 'Responsive Table Alternative', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H49" s="6" t="inlineStr">
         <is>
-          <t>Each mobile row must show label and value.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Table Alternative'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
@@ -3108,12 +3108,12 @@
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>Define spacing variables on :root.</t>
+          <t>Inspect the provided markup for 'Scalable Spacing System', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H50" s="4" t="inlineStr">
         <is>
-          <t>Avoid hardcoding repeated pixel spacing.</t>
+          <t>Do not change the provided HTML structure for 'Scalable Spacing System'. The submitted CSS must match the sample output for question 49 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -3161,12 +3161,12 @@
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Use flex or grid with a breakpoint.</t>
+          <t>Start from the smallest screen layout for 'Accessible Responsive Footer', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>Link tap targets must be at least 44px high on mobile.</t>
+          <t>Do not change the provided HTML structure for 'Accessible Responsive Footer'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3214,12 +3214,12 @@
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>Use @media (max-width: 600px).</t>
+          <t>Start from the smallest screen layout for 'Write Your First Media Query', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H52" s="4" t="inlineStr">
         <is>
-          <t>Mobile card must fit within the viewport.</t>
+          <t>Do not change the provided HTML structure for 'Write Your First Media Query'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I52" s="4" t="inlineStr">
@@ -3267,12 +3267,12 @@
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>Put mobile styles outside the media query.</t>
+          <t>Start from the smallest screen layout for 'Use Mobile First CSS', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>Desktop rules must use min-width.</t>
+          <t>Do not change the provided HTML structure for 'Use Mobile First CSS'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -3320,12 +3320,12 @@
       </c>
       <c r="G54" s="4" t="inlineStr">
         <is>
-          <t>Set body font size and paragraph max-width.</t>
+          <t>Start from the smallest screen layout for 'Make Text Responsive', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H54" s="4" t="inlineStr">
         <is>
-          <t>Do not use viewport-width font sizing.</t>
+          <t>Do not change the provided HTML structure for 'Make Text Responsive'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I54" s="4" t="inlineStr">
@@ -3373,12 +3373,12 @@
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>Use flex-direction and a breakpoint.</t>
+          <t>Start from the smallest screen layout for 'Responsive Button Group', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>Buttons must remain easy to tap on mobile.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Button Group'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -3426,12 +3426,12 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>Use display none in a media query.</t>
+          <t>Start from the smallest screen layout for 'Hide Decorative Content on Mobile', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
         <is>
-          <t>Do not hide important content.</t>
+          <t>Do not change the provided HTML structure for 'Hide Decorative Content on Mobile'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I56" s="4" t="inlineStr">
@@ -3479,12 +3479,12 @@
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>Use grid and a min-width breakpoint.</t>
+          <t>Start from the smallest screen layout for 'Responsive Pricing Cards', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>Cards must not overflow on mobile.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Pricing Cards'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
@@ -3532,12 +3532,12 @@
       </c>
       <c r="G58" s="4" t="inlineStr">
         <is>
-          <t>Use width 100% and height auto.</t>
+          <t>Inspect the provided markup for 'Fluid Image Banner', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H58" s="4" t="inlineStr">
         <is>
-          <t>Image must not appear stretched.</t>
+          <t>Do not change the provided HTML structure for 'Fluid Image Banner'. The submitted CSS must match the sample output for question 57 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I58" s="4" t="inlineStr">
@@ -3585,12 +3585,12 @@
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>Use CSS variables or media queries.</t>
+          <t>Start from the smallest screen layout for 'Responsive Spacing Tokens', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>Mobile spacing must remain compact.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Spacing Tokens'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -3638,12 +3638,12 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>Use grid or flex with a breakpoint.</t>
+          <t>Start from the smallest screen layout for 'Responsive Sidebar Collapse', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H60" s="4" t="inlineStr">
         <is>
-          <t>Content must appear below navigation on mobile.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Sidebar Collapse'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I60" s="4" t="inlineStr">
@@ -3691,12 +3691,12 @@
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>Check fixed widths and use max-width.</t>
+          <t>Inspect the provided markup for 'Prevent Horizontal Scroll', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>Page width must not exceed viewport width.</t>
+          <t>Do not change the provided HTML structure for 'Prevent Horizontal Scroll'. The submitted CSS must match the sample output for question 60 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -3744,12 +3744,12 @@
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Use spacing, text, border, and shadow utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Profile Card': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H62" s="4" t="inlineStr">
         <is>
-          <t>Do not write custom CSS.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Profile Card'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I62" s="4" t="inlineStr">
@@ -3796,12 +3796,12 @@
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>Use md:flex and gap utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Responsive Navbar': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H63" s="6" t="inlineStr">
         <is>
-          <t>Mobile layout must remain readable.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Responsive Navbar'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -3848,12 +3848,12 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>Use grid-cols-1, md:grid-cols-2, and lg:grid-cols-3.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Course Grid': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H64" s="4" t="inlineStr">
         <is>
-          <t>Cards must have equal spacing.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Course Grid'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
@@ -3900,12 +3900,12 @@
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>Use hover:, focus:, and ring utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Button States': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>Buttons must include visible focus styling.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Button States'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -3952,12 +3952,12 @@
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>Apply classes directly to labels and inputs.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Form Panel': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H66" s="4" t="inlineStr">
         <is>
-          <t>Inputs must be full width.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Form Panel'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -4004,12 +4004,12 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>Use min-h-screen, w-64, and flex utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Sidebar Layout': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>Sidebar should remain left aligned on desktop.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Sidebar Layout'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -4056,12 +4056,12 @@
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>Assume the theme has brand colors configured.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Theme Color Usage': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H68" s="4" t="inlineStr">
         <is>
-          <t>Use brand utility names consistently.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Theme Color Usage'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
@@ -4108,12 +4108,12 @@
       </c>
       <c r="G69" s="6" t="inlineStr">
         <is>
-          <t>Map spacing values to closest Tailwind scale.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Spacing System': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H69" s="6" t="inlineStr">
         <is>
-          <t>Do not use arbitrary values unless necessary.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Spacing System'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -4160,12 +4160,12 @@
       </c>
       <c r="G70" s="4" t="inlineStr">
         <is>
-          <t>Use grid utilities and semantic text sizes.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Dashboard Widgets': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H70" s="4" t="inlineStr">
         <is>
-          <t>Widgets must align in a responsive grid.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Dashboard Widgets'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
@@ -4212,12 +4212,12 @@
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>Use shared base classes and variant classes.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Production Component': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>Each variant must have accessible contrast.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Production Component'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4264,12 +4264,12 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>Use text, font, leading, and color utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Text Styling': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H72" s="4" t="inlineStr">
         <is>
-          <t>Do not write custom CSS.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Text Styling'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -4316,12 +4316,12 @@
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>Use p, m, mt, and gap utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Spacing Practice': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>Avoid arbitrary values.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Spacing Practice'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4368,12 +4368,12 @@
       </c>
       <c r="G74" s="4" t="inlineStr">
         <is>
-          <t>Use min-h-screen, flex, items-center, and justify-center.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Flex Centering': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H74" s="4" t="inlineStr">
         <is>
-          <t>Do not use custom CSS.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Flex Centering'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -4420,12 +4420,12 @@
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>Use rounded-full and px/py utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Color Badges': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>Badge colors must be readable.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Color Badges'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
@@ -4472,12 +4472,12 @@
       </c>
       <c r="G76" s="4" t="inlineStr">
         <is>
-          <t>Use border, rounded, p, and shadow utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Border Card': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H76" s="4" t="inlineStr">
         <is>
-          <t>Card must have visible spacing.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Border Card'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
@@ -4524,12 +4524,12 @@
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>Use text-2xl and md:text-4xl style classes.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Responsive Text': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>Base class must support mobile first.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Responsive Text'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4576,12 +4576,12 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>Use grid, grid-cols-1, md:grid-cols-2, and gap.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Grid Basics': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H78" s="4" t="inlineStr">
         <is>
-          <t>No custom media query allowed.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Grid Basics'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I78" s="4" t="inlineStr">
@@ -4628,12 +4628,12 @@
       </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>Use focus:ring and focus:border utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Form Inputs': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>Focus state must be visible.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Form Inputs'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -4680,12 +4680,12 @@
       </c>
       <c r="G80" s="4" t="inlineStr">
         <is>
-          <t>Use hover: utilities.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Button Hover': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H80" s="4" t="inlineStr">
         <is>
-          <t>Button text must remain readable on hover.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Button Hover'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I80" s="4" t="inlineStr">
@@ -4732,12 +4732,12 @@
       </c>
       <c r="G81" s="6" t="inlineStr">
         <is>
-          <t>Use utility classes only.</t>
+          <t>Use Tailwind utilities that directly express the target for 'Tailwind Simple Alert': spacing, color, layout, and state classes should be visible in the class attribute without adding a custom CSS file.</t>
         </is>
       </c>
       <c r="H81" s="6" t="inlineStr">
         <is>
-          <t>Alert must include comfortable padding.</t>
+          <t>Do not change the provided HTML structure for 'Tailwind Simple Alert'. Use Tailwind utility classes only; do not add a separate CSS selector, inline style block, or arbitrary value unless the question explicitly requires it.</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -4784,12 +4784,12 @@
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>Use transition and transform properties.</t>
+          <t>Implement the visible UI state for 'Hoverable Dashboard Card' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H82" s="4" t="inlineStr">
         <is>
-          <t>Hover effect must be subtle and not shift layout.</t>
+          <t>Do not change the provided HTML structure for 'Hoverable Dashboard Card'. The interaction effect must not resize surrounding layout or cause nearby text, buttons, or cards to jump.</t>
         </is>
       </c>
       <c r="I82" s="4" t="inlineStr">
@@ -4837,12 +4837,12 @@
       </c>
       <c r="G83" s="6" t="inlineStr">
         <is>
-          <t>Use pseudo-classes and transitions.</t>
+          <t>Inspect the provided markup for 'Animated Submit Button', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>Disabled state must look inactive and block pointer styling.</t>
+          <t>Do not change the provided HTML structure for 'Animated Submit Button'. The submitted CSS must match the sample output for question 82 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -4890,12 +4890,12 @@
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Use gradients and keyframe animation.</t>
+          <t>Implement the visible UI state for 'Skeleton Loading Card' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H84" s="4" t="inlineStr">
         <is>
-          <t>Animation should be smooth and not distract users.</t>
+          <t>Do not change the provided HTML structure for 'Skeleton Loading Card'. Animation duration should stay under 500ms for entrance effects, and layout-changing properties such as width, height, top, or left should be avoided.</t>
         </is>
       </c>
       <c r="I84" s="4" t="inlineStr">
@@ -4943,12 +4943,12 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>Use classes for active state and pseudo-classes for interactions.</t>
+          <t>Inspect the provided markup for 'Sidebar Navigation States', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H85" s="6" t="inlineStr">
         <is>
-          <t>Active state must differ from hover state.</t>
+          <t>Do not change the provided HTML structure for 'Sidebar Navigation States'. The submitted CSS must match the sample output for question 84 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I85" s="6" t="inlineStr">
@@ -4996,12 +4996,12 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>Use :focus, :valid, and :invalid selectors.</t>
+          <t>Style the form controls for 'Interactive Form Feedback' in their normal and focus states; labels, inputs, helper text, and buttons should remain aligned and readable.</t>
         </is>
       </c>
       <c r="H86" s="4" t="inlineStr">
         <is>
-          <t>Invalid state must not rely only on color.</t>
+          <t>Do not change the provided HTML structure for 'Interactive Form Feedback'. Inputs must remain keyboard focusable, labels must remain visible, and focus styling must not be removed.</t>
         </is>
       </c>
       <c r="I86" s="4" t="inlineStr">
@@ -5049,12 +5049,12 @@
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>Use heading, value, and helper text styles.</t>
+          <t>Inspect the provided markup for 'Card Widget Hierarchy', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>The metric value must be the most prominent element.</t>
+          <t>Do not change the provided HTML structure for 'Card Widget Hierarchy'. The submitted CSS must match the sample output for question 86 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -5102,12 +5102,12 @@
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>Use @keyframes and animation properties.</t>
+          <t>Inspect the provided markup for 'Fade In Content Section', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H88" s="4" t="inlineStr">
         <is>
-          <t>Animation duration must be under 500ms.</t>
+          <t>Do not change the provided HTML structure for 'Fade In Content Section'. Animation duration should stay under 500ms for entrance effects, and layout-changing properties such as width, height, top, or left should be avoided.</t>
         </is>
       </c>
       <c r="I88" s="4" t="inlineStr">
@@ -5155,12 +5155,12 @@
       </c>
       <c r="G89" s="6" t="inlineStr">
         <is>
-          <t>Use position and opacity transitions.</t>
+          <t>Inspect the provided markup for 'Accessible Tooltip Styling', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H89" s="6" t="inlineStr">
         <is>
-          <t>Tooltip must work with keyboard focus.</t>
+          <t>Do not change the provided HTML structure for 'Accessible Tooltip Styling'. The submitted CSS must match the sample output for question 88 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -5208,12 +5208,12 @@
       </c>
       <c r="G90" s="4" t="inlineStr">
         <is>
-          <t>Use transform, opacity, and transition.</t>
+          <t>Set the correct positioning context for 'Interactive Modal Motion' before applying top/right/bottom/left or z-index values, then verify the layer appears exactly where the output page shows it.</t>
         </is>
       </c>
       <c r="H90" s="4" t="inlineStr">
         <is>
-          <t>Respect reduced motion with a media query.</t>
+          <t>Do not change the provided HTML structure for 'Interactive Modal Motion'. The overlay must sit below the dialog, the dialog must remain visible above the overlay, and the page content must not visually cover the modal.</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr">
@@ -5261,12 +5261,12 @@
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>Use layout, spacing, and subtle color hierarchy.</t>
+          <t>Inspect the provided markup for 'Empty State Panel', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>The action button must remain visually prominent.</t>
+          <t>Do not change the provided HTML structure for 'Empty State Panel'. The submitted CSS must match the sample output for question 90 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
@@ -5314,12 +5314,12 @@
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>Use transition on the button.</t>
+          <t>Implement the visible UI state for 'Button Hover Feedback' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H92" s="4" t="inlineStr">
         <is>
-          <t>Hover must not change button size.</t>
+          <t>Do not change the provided HTML structure for 'Button Hover Feedback'. The interaction effect must not resize surrounding layout or cause nearby text, buttons, or cards to jump.</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
@@ -5367,12 +5367,12 @@
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>Use box-shadow and transition.</t>
+          <t>Implement the visible UI state for 'Card Hover Shadow' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>The card must not jump on hover.</t>
+          <t>Do not change the provided HTML structure for 'Card Hover Shadow'. The interaction effect must not resize surrounding layout or cause nearby text, buttons, or cards to jump.</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5420,12 +5420,12 @@
       </c>
       <c r="G94" s="4" t="inlineStr">
         <is>
-          <t>Use :focus and outline or box-shadow.</t>
+          <t>Style the form controls for 'Input Focus State' in their normal and focus states; labels, inputs, helper text, and buttons should remain aligned and readable.</t>
         </is>
       </c>
       <c r="H94" s="4" t="inlineStr">
         <is>
-          <t>Do not remove focus feedback.</t>
+          <t>Do not change the provided HTML structure for 'Input Focus State'. Inputs must remain keyboard focusable, labels must remain visible, and focus styling must not be removed.</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
@@ -5473,12 +5473,12 @@
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>Use opacity and cursor styles.</t>
+          <t>Implement the visible UI state for 'Simple Loading State' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H95" s="6" t="inlineStr">
         <is>
-          <t>Button must look disabled.</t>
+          <t>Do not change the provided HTML structure for 'Simple Loading State'. Animation duration should stay under 500ms for entrance effects, and layout-changing properties such as width, height, top, or left should be avoided.</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -5526,12 +5526,12 @@
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Use an active class.</t>
+          <t>Implement the visible UI state for 'Create Active Menu Item' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H96" s="4" t="inlineStr">
         <is>
-          <t>Active state must be visually stronger than hover.</t>
+          <t>Do not change the provided HTML structure for 'Create Active Menu Item'. The submitted CSS must match the sample output for question 95 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr">
@@ -5579,12 +5579,12 @@
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>Use @keyframes and animation.</t>
+          <t>Inspect the provided markup for 'Smooth Fade Effect', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>Animation must finish quickly.</t>
+          <t>Do not change the provided HTML structure for 'Smooth Fade Effect'. Animation duration should stay under 500ms for entrance effects, and layout-changing properties such as width, height, top, or left should be avoided.</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -5632,12 +5632,12 @@
       </c>
       <c r="G98" s="4" t="inlineStr">
         <is>
-          <t>Use position absolute and opacity.</t>
+          <t>Inspect the provided markup for 'Icon Button Tooltip', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H98" s="4" t="inlineStr">
         <is>
-          <t>Tooltip text must be readable.</t>
+          <t>Do not change the provided HTML structure for 'Icon Button Tooltip'. The submitted CSS must match the sample output for question 97 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I98" s="4" t="inlineStr">
@@ -5685,12 +5685,12 @@
       </c>
       <c r="G99" s="6" t="inlineStr">
         <is>
-          <t>Use spacing and visual hierarchy.</t>
+          <t>Inspect the provided markup for 'Design Empty State', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>Primary action must be easy to find.</t>
+          <t>Do not change the provided HTML structure for 'Design Empty State'. The submitted CSS must match the sample output for question 98 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -5738,12 +5738,12 @@
       </c>
       <c r="G100" s="4" t="inlineStr">
         <is>
-          <t>Use color, spacing, and helper text.</t>
+          <t>Inspect the provided markup for 'Style Error Message', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H100" s="4" t="inlineStr">
         <is>
-          <t>Do not rely on color alone.</t>
+          <t>Do not change the provided HTML structure for 'Style Error Message'. The submitted CSS must match the sample output for question 99 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I100" s="4" t="inlineStr">
@@ -5791,12 +5791,12 @@
       </c>
       <c r="G101" s="6" t="inlineStr">
         <is>
-          <t>Use transition-property and duration.</t>
+          <t>Implement the visible UI state for 'Create Transitioned Panel' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>Effect must remain subtle.</t>
+          <t>Do not change the provided HTML structure for 'Create Transitioned Panel'. The interaction effect must not resize surrounding layout or cause nearby text, buttons, or cards to jump.</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5844,12 +5844,12 @@
       </c>
       <c r="G102" s="4" t="inlineStr">
         <is>
-          <t>Separate base class from variant classes.</t>
+          <t>Create reusable styling for 'Reusable Component Classes' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H102" s="4" t="inlineStr">
         <is>
-          <t>Do not duplicate shared button declarations.</t>
+          <t>Do not change the provided HTML structure for 'Reusable Component Classes'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I102" s="4" t="inlineStr">
@@ -5896,12 +5896,12 @@
       </c>
       <c r="G103" s="6" t="inlineStr">
         <is>
-          <t>Use comments only for major sections.</t>
+          <t>Create reusable styling for 'Organized CSS Structure' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>Keep selectors readable and avoid deep nesting.</t>
+          <t>Do not change the provided HTML structure for 'Organized CSS Structure'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -5948,12 +5948,12 @@
       </c>
       <c r="G104" s="4" t="inlineStr">
         <is>
-          <t>Define tokens on :root and override them with a theme class.</t>
+          <t>Create reusable styling for 'CSS Variables Theme' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H104" s="4" t="inlineStr">
         <is>
-          <t>Components must use variables instead of hardcoded colors.</t>
+          <t>Do not change the provided HTML structure for 'CSS Variables Theme'. Repeated colors, spacing, or radius values must be represented with CSS custom properties and reused in component rules.</t>
         </is>
       </c>
       <c r="I104" s="4" t="inlineStr">
@@ -6000,12 +6000,12 @@
       </c>
       <c r="G105" s="6" t="inlineStr">
         <is>
-          <t>Choose foreground/background pairs with clear contrast.</t>
+          <t>Choose foreground, background, and border colors for 'Accessible Contrast Fix' so every state is visually distinct and the text stays readable.</t>
         </is>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>Do not reduce font size to solve layout issues.</t>
+          <t>Do not change the provided HTML structure for 'Accessible Contrast Fix'. Each visual state must include readable text contrast and at least one non-color cue such as a border, label, icon, or spacing difference.</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -6052,12 +6052,12 @@
       </c>
       <c r="G106" s="4" t="inlineStr">
         <is>
-          <t>Create predictable classes for each state.</t>
+          <t>Style the form controls for 'Production Form Component' in their normal and focus states; labels, inputs, helper text, and buttons should remain aligned and readable.</t>
         </is>
       </c>
       <c r="H106" s="4" t="inlineStr">
         <is>
-          <t>Error text must be visible and associated with the field visually.</t>
+          <t>Do not change the provided HTML structure for 'Production Form Component'. Inputs must remain keyboard focusable, labels must remain visible, and focus styling must not be removed.</t>
         </is>
       </c>
       <c r="I106" s="4" t="inlineStr">
@@ -6104,12 +6104,12 @@
       </c>
       <c r="G107" s="6" t="inlineStr">
         <is>
-          <t>Prefer CSS gradients or optimized reusable assets.</t>
+          <t>Inspect the provided markup for 'Optimize CSS Asset Usage', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H107" s="6" t="inlineStr">
         <is>
-          <t>Do not remove required brand visuals.</t>
+          <t>Do not change the provided HTML structure for 'Optimize CSS Asset Usage'. The submitted CSS must match the sample output for question 106 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I107" s="6" t="inlineStr">
@@ -6156,12 +6156,12 @@
       </c>
       <c r="G108" s="4" t="inlineStr">
         <is>
-          <t>Use a consistent prefix or BEM-style naming.</t>
+          <t>Create reusable styling for 'Component Scoped Naming' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H108" s="4" t="inlineStr">
         <is>
-          <t>Class names must communicate component ownership.</t>
+          <t>Do not change the provided HTML structure for 'Component Scoped Naming'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I108" s="4" t="inlineStr">
@@ -6208,12 +6208,12 @@
       </c>
       <c r="G109" s="6" t="inlineStr">
         <is>
-          <t>Use reusable layout classes and responsive rules.</t>
+          <t>Inspect the provided markup for 'Production Dashboard Layout', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>The shell must remain usable on mobile.</t>
+          <t>Do not change the provided HTML structure for 'Production Dashboard Layout'. The submitted CSS must match the sample output for question 108 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -6260,12 +6260,12 @@
       </c>
       <c r="G110" s="4" t="inlineStr">
         <is>
-          <t>Use semantic selectors carefully with classes for components.</t>
+          <t>Inspect the provided markup for 'Semantic UI Styling', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H110" s="4" t="inlineStr">
         <is>
-          <t>Do not remove outlines or hide labels.</t>
+          <t>Do not change the provided HTML structure for 'Semantic UI Styling'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I110" s="4" t="inlineStr">
@@ -6312,12 +6312,12 @@
       </c>
       <c r="G111" s="6" t="inlineStr">
         <is>
-          <t>Animate transform and opacity only where possible.</t>
+          <t>Style the form controls for 'Performance Friendly Animation' in their normal and focus states; labels, inputs, helper text, and buttons should remain aligned and readable.</t>
         </is>
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>Avoid animating width, height, top, or left.</t>
+          <t>Do not change the provided HTML structure for 'Performance Friendly Animation'. Inputs must remain keyboard focusable, labels must remain visible, and focus styling must not be removed.</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -6364,12 +6364,12 @@
       </c>
       <c r="G112" s="4" t="inlineStr">
         <is>
-          <t>Use :root custom properties.</t>
+          <t>Create reusable styling for 'Create Design Tokens' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H112" s="4" t="inlineStr">
         <is>
-          <t>Components must reference the variables.</t>
+          <t>Do not change the provided HTML structure for 'Create Design Tokens'. Repeated colors, spacing, or radius values must be represented with CSS custom properties and reused in component rules.</t>
         </is>
       </c>
       <c r="I112" s="4" t="inlineStr">
@@ -6416,12 +6416,12 @@
       </c>
       <c r="G113" s="6" t="inlineStr">
         <is>
-          <t>Use a shared base class and variants.</t>
+          <t>Create reusable styling for 'Reusable Button System' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>Avoid duplicate declarations.</t>
+          <t>Do not change the provided HTML structure for 'Reusable Button System'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
@@ -6468,12 +6468,12 @@
       </c>
       <c r="G114" s="4" t="inlineStr">
         <is>
-          <t>Use component-based class names.</t>
+          <t>Create reusable styling for 'Reusable Card Component' by separating shared base rules from component-specific variants and using clear class names.</t>
         </is>
       </c>
       <c r="H114" s="4" t="inlineStr">
         <is>
-          <t>Class names must be predictable.</t>
+          <t>Do not change the provided HTML structure for 'Reusable Card Component'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I114" s="4" t="inlineStr">
@@ -6520,12 +6520,12 @@
       </c>
       <c r="G115" s="6" t="inlineStr">
         <is>
-          <t>Use :focus-visible.</t>
+          <t>Implement the visible UI state for 'Accessible Focus Styles' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H115" s="6" t="inlineStr">
         <is>
-          <t>Do not set outline to none without replacement.</t>
+          <t>Do not change the provided HTML structure for 'Accessible Focus Styles'. The submitted CSS must match the sample output for question 114 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I115" s="6" t="inlineStr">
@@ -6572,12 +6572,12 @@
       </c>
       <c r="G116" s="4" t="inlineStr">
         <is>
-          <t>Use short section comments.</t>
+          <t>Inspect the provided markup for 'Organize CSS File Sections', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H116" s="4" t="inlineStr">
         <is>
-          <t>Do not change behavior while organizing.</t>
+          <t>Do not change the provided HTML structure for 'Organize CSS File Sections'. The submitted CSS must match the sample output for question 115 without using JavaScript, external images, or !important.</t>
         </is>
       </c>
       <c r="I116" s="4" t="inlineStr">
@@ -6624,12 +6624,12 @@
       </c>
       <c r="G117" s="6" t="inlineStr">
         <is>
-          <t>Use classes for component-specific styling.</t>
+          <t>Inspect the provided markup for 'Use Semantic Layout Classes', identify the key class names, and write the smallest set of CSS rules needed to reproduce the linked sample output.</t>
         </is>
       </c>
       <c r="H117" s="6" t="inlineStr">
         <is>
-          <t>Do not depend only on tag selectors.</t>
+          <t>Do not change the provided HTML structure for 'Use Semantic Layout Classes'. Class names must be predictable and reusable; do not rely on deeply nested selectors or remove semantic accessibility behavior.</t>
         </is>
       </c>
       <c r="I117" s="6" t="inlineStr">
@@ -6676,12 +6676,12 @@
       </c>
       <c r="G118" s="4" t="inlineStr">
         <is>
-          <t>Create variables and reuse them.</t>
+          <t>Choose foreground, background, and border colors for 'Reduce Repeated Colors' so every state is visually distinct and the text stays readable.</t>
         </is>
       </c>
       <c r="H118" s="4" t="inlineStr">
         <is>
-          <t>Keep the visual result unchanged.</t>
+          <t>Do not change the provided HTML structure for 'Reduce Repeated Colors'. Each visual state must include readable text contrast and at least one non-color cue such as a border, label, icon, or spacing difference.</t>
         </is>
       </c>
       <c r="I118" s="4" t="inlineStr">
@@ -6728,12 +6728,12 @@
       </c>
       <c r="G119" s="6" t="inlineStr">
         <is>
-          <t>Avoid animating layout properties.</t>
+          <t>Implement the visible UI state for 'Safe Animation Choices' with pseudo-classes, transitions, transforms, opacity, or keyframes while keeping the base state clear.</t>
         </is>
       </c>
       <c r="H119" s="6" t="inlineStr">
         <is>
-          <t>Do not animate width or height.</t>
+          <t>Do not change the provided HTML structure for 'Safe Animation Choices'. Animation duration should stay under 500ms for entrance effects, and layout-changing properties such as width, height, top, or left should be avoided.</t>
         </is>
       </c>
       <c r="I119" s="6" t="inlineStr">
@@ -6780,12 +6780,12 @@
       </c>
       <c r="G120" s="4" t="inlineStr">
         <is>
-          <t>Use a breakpoint to change layout.</t>
+          <t>Start from the smallest screen layout for 'Responsive Production Shell', then add the required breakpoint rule so the sample output changes layout without horizontal scrolling.</t>
         </is>
       </c>
       <c r="H120" s="4" t="inlineStr">
         <is>
-          <t>Mobile layout must remain usable.</t>
+          <t>Do not change the provided HTML structure for 'Responsive Production Shell'. The final page must work at 375px and 1024px widths, must not create horizontal scroll, and must use the breakpoint behavior requested by the prompt.</t>
         </is>
       </c>
       <c r="I120" s="4" t="inlineStr">
@@ -6832,12 +6832,12 @@
       </c>
       <c r="G121" s="6" t="inlineStr">
         <is>
-          <t>Use icons, borders, or labels in addition to color.</t>
+          <t>Choose foreground, background, and border colors for 'Accessible Color States' so every state is visually distinct and the text stays readable.</t>
         </is>
       </c>
       <c r="H121" s="6" t="inlineStr">
         <is>
-          <t>Contrast must be readable.</t>
+          <t>Do not change the provided HTML structure for 'Accessible Color States'. Each visual state must include readable text contrast and at least one non-color cue such as a border, label, icon, or spacing difference.</t>
         </is>
       </c>
       <c r="I121" s="6" t="inlineStr">

</xml_diff>